<commit_message>
chore(data): batch update intraday supervisor - 08:02:17
</commit_message>
<xml_diff>
--- a/data/dim_supervisor.xlsx
+++ b/data/dim_supervisor.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B140"/>
+  <dimension ref="A1:B141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1792,39 +1792,49 @@
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>SUPERVISOR FARMA PE</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
+        <v>147</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
         <v>9999</v>
       </c>
-      <c r="B140" t="inlineStr">
+      <c r="B141" t="inlineStr">
         <is>
           <t>TODOS OS SUPERVISORES</t>
         </is>

</xml_diff>